<commit_message>
roll port tested ok
</commit_message>
<xml_diff>
--- a/tests/testthat/testdata/transaction_cost_calc.xlsx
+++ b/tests/testthat/testdata/transaction_cost_calc.xlsx
@@ -1,26 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo.fonteles\OneDrive - Sicoob\Renda Variável\Multifatorial 3.0\factoRverse\tests\testthat\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{A2D53C65-09A8-493D-B5ED-C26A20314A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADCF3DFA-C9C7-4B81-B0A3-84EDA074AB1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-1065" windowWidth="20730" windowHeight="11160" xr2:uid="{0D95CC1D-80FD-4D8F-96FF-C13E93866E2C}"/>
+    <workbookView xWindow="-20610" yWindow="-1065" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{0D95CC1D-80FD-4D8F-96FF-C13E93866E2C}"/>
   </bookViews>
   <sheets>
-    <sheet name="trans" sheetId="1" r:id="rId1"/>
+    <sheet name="transaction_cost" sheetId="1" r:id="rId1"/>
+    <sheet name="full_roll_port_3_periods" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
   <si>
     <t>id</t>
   </si>
@@ -98,15 +112,42 @@
   </si>
   <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>SW Port at  2001-06-15</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>Updated</t>
+  </si>
+  <si>
+    <t>Wx(1+R)</t>
+  </si>
+  <si>
+    <t>15/07/2001</t>
+  </si>
+  <si>
+    <t>BOP_W</t>
+  </si>
+  <si>
+    <t>EOP_W</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.000000000000000%"/>
+    <numFmt numFmtId="169" formatCode="0.0000%"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -244,7 +285,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -422,6 +463,18 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -587,13 +640,45 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="33" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="34" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="33" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Ênfase1" xfId="21" builtinId="30" customBuiltin="1"/>
@@ -974,6 +1059,7 @@
   <dimension ref="A1:R14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="4" max="4" width="10.42578125" customWidth="1"/>
     <col min="15" max="15" width="9.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19" bestFit="1" customWidth="1"/>
   </cols>
@@ -1054,34 +1140,34 @@
         <v>5.4051600740000003</v>
       </c>
       <c r="J2">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K2">
         <f>E2-J2</f>
-        <v>0.54800595112359296</v>
+        <v>0.34800595112359295</v>
       </c>
       <c r="L2">
         <f>K2*$L$8</f>
-        <v>5.4800595112359298</v>
+        <v>0.34800595112359295</v>
       </c>
       <c r="M2" s="4">
         <f>L2/G2</f>
-        <v>0.14099294391715053</v>
+        <v>8.9536223920563453E-3</v>
       </c>
       <c r="N2">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="O2">
         <f>ABS(L2*0.07)</f>
-        <v>0.38360416578651513</v>
+        <v>2.4360416578651508E-2</v>
       </c>
       <c r="P2">
-        <f>M2^N2*I2/2</f>
-        <v>2.2217659279333346</v>
+        <f>ABS(M2)^N2*I2/2</f>
+        <v>0.25572780547838786</v>
       </c>
       <c r="R2">
         <f>M2^N2*I2/2</f>
-        <v>2.2217659279333346</v>
+        <v>0.25572780547838786</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -1113,34 +1199,34 @@
         <v>0.25392852100000002</v>
       </c>
       <c r="J3">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K3">
         <f>E3-J3</f>
-        <v>0.16283255805920199</v>
+        <v>-3.7167441940798018E-2</v>
       </c>
       <c r="L3">
         <f>K3*$L$8</f>
-        <v>1.62832558059202</v>
+        <v>-3.7167441940798018E-2</v>
       </c>
       <c r="M3" s="4">
         <f t="shared" ref="M3:M6" si="0">L3/G3</f>
-        <v>0.10408278184177187</v>
+        <v>-2.3757476988934315E-3</v>
       </c>
       <c r="N3">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="O3">
         <f>ABS(L3*0.07)</f>
-        <v>0.11398279064144141</v>
+        <v>2.6017209358558616E-3</v>
       </c>
       <c r="P3">
-        <f t="shared" ref="P3:P6" si="1">M3^N3*I3/2</f>
-        <v>0.10125567580480922</v>
-      </c>
-      <c r="R3">
+        <f>ABS(M3)^N3*I3/2</f>
+        <v>6.1884465764165883E-3</v>
+      </c>
+      <c r="R3" t="e">
         <f>M3^N3*I3/2</f>
-        <v>0.10125567580480922</v>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
@@ -1172,34 +1258,34 @@
         <v>4.4926513650000004</v>
       </c>
       <c r="J4">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K4">
         <f>E4-J4</f>
-        <v>0.126328932758003</v>
+        <v>-7.3671067241997013E-2</v>
       </c>
       <c r="L4">
         <f>K4*$L$8</f>
-        <v>1.2632893275800301</v>
+        <v>-7.3671067241997013E-2</v>
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>8.1026217637995585E-2</v>
+        <v>-4.725194615083376E-3</v>
       </c>
       <c r="N4">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O4">
         <f>ABS(L4*0.07)</f>
-        <v>8.843025293060211E-2</v>
+        <v>5.1569747069397914E-3</v>
       </c>
       <c r="P4">
-        <f t="shared" si="1"/>
-        <v>1.1984753722078016</v>
-      </c>
-      <c r="R4">
+        <f>ABS(M4)^N4*I4/2</f>
+        <v>0.15441254203649388</v>
+      </c>
+      <c r="R4" t="e">
         <f>M4^N4*I4/2</f>
-        <v>1.1984753722078016</v>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1231,34 +1317,34 @@
         <v>1.6131663460000001</v>
       </c>
       <c r="J5">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K5">
         <f>E5-J5</f>
-        <v>0.16283255805920199</v>
+        <v>-3.7167441940798018E-2</v>
       </c>
       <c r="L5">
-        <f t="shared" ref="L3:L6" si="2">K5*$L$8</f>
-        <v>1.62832558059202</v>
+        <f t="shared" ref="L5:L6" si="1">K5*$L$8</f>
+        <v>-3.7167441940798018E-2</v>
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>6.2570517339539847E-2</v>
+        <v>-1.4282070478666288E-3</v>
       </c>
       <c r="N5">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O5">
         <f>ABS(L5*0.07)</f>
-        <v>0.11398279064144141</v>
+        <v>2.6017209358558616E-3</v>
       </c>
       <c r="P5">
-        <f t="shared" si="1"/>
-        <v>0.40340529459990138</v>
-      </c>
-      <c r="R5">
+        <f>ABS(M5)^N5*I5/2</f>
+        <v>3.0482090168348262E-2</v>
+      </c>
+      <c r="R5" t="e">
         <f>M5^N5*I5/2</f>
-        <v>0.40340529459990138</v>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
@@ -1290,39 +1376,39 @@
         <v>3.0529088560000002</v>
       </c>
       <c r="J6">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="K6">
         <f>E6-J6</f>
-        <v>0</v>
+        <v>-0.2</v>
       </c>
       <c r="L6">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>-0.2</v>
       </c>
       <c r="M6" s="5">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-1.2794945451993585E-2</v>
       </c>
       <c r="N6">
         <v>0.5</v>
       </c>
       <c r="O6">
         <f>ABS(L6*0.07)</f>
-        <v>0</v>
+        <v>1.4000000000000002E-2</v>
       </c>
       <c r="P6">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="R6">
+        <f>ABS(M6)^N6*I6/2</f>
+        <v>0.17266450280771806</v>
+      </c>
+      <c r="R6" t="e">
         <f>M6^N6*I6/2</f>
-        <v>0</v>
+        <v>#NUM!</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="L8">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
@@ -1345,6 +1431,290 @@
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P14" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F36494F6-E719-42C3-AE2F-526661CDA40A}">
+  <dimension ref="B2:N1048576"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B2" s="1">
+        <v>37057</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+    </row>
+    <row r="3" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="D3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="N3" s="6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0.54800599999999999</v>
+      </c>
+      <c r="E4" s="9">
+        <v>1.6764270000000001E-2</v>
+      </c>
+      <c r="F4" s="2">
+        <f>D4*(1+E4)</f>
+        <v>0.55719292054561997</v>
+      </c>
+      <c r="G4" s="8">
+        <f>F4/$F$8</f>
+        <v>0.54998005054117849</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="16">
+        <f>G4</f>
+        <v>0.54998005054117849</v>
+      </c>
+      <c r="K4" s="18"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="8">
+        <f>K4*(1+L4)</f>
+        <v>0</v>
+      </c>
+      <c r="N4" s="8">
+        <f>M4/$M$9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="8">
+        <v>0.16283259999999999</v>
+      </c>
+      <c r="E5" s="9">
+        <v>1.9005850000000001E-2</v>
+      </c>
+      <c r="F5" s="2">
+        <f t="shared" ref="F5:G7" si="0">D5*(1+E5)</f>
+        <v>0.16592737197071</v>
+      </c>
+      <c r="G5" s="8">
+        <f>F5/$F$8</f>
+        <v>0.16377943986304544</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="J5" s="14">
+        <v>0</v>
+      </c>
+      <c r="K5" s="17">
+        <v>0</v>
+      </c>
+      <c r="L5" s="9">
+        <v>1.3249703999999999E-2</v>
+      </c>
+      <c r="M5" s="8">
+        <f t="shared" ref="M5:M8" si="1">K5*(1+L5)</f>
+        <v>0</v>
+      </c>
+      <c r="N5" s="8">
+        <f t="shared" ref="N5:N8" si="2">M5/$M$9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" s="8">
+        <v>0.12632889999999999</v>
+      </c>
+      <c r="E6" s="9">
+        <v>-1.2873559999999999E-2</v>
+      </c>
+      <c r="F6" s="2">
+        <f t="shared" si="0"/>
+        <v>0.12470259732611599</v>
+      </c>
+      <c r="G6" s="8">
+        <f>F6/$F$8</f>
+        <v>0.12308832049207313</v>
+      </c>
+      <c r="I6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J6" s="12">
+        <f>G5</f>
+        <v>0.16377943986304544</v>
+      </c>
+      <c r="K6" s="8">
+        <f>J6/SUM($J$5:$J$8)</f>
+        <v>0.3639381766519485</v>
+      </c>
+      <c r="L6" s="9">
+        <v>-9.0214219999999994E-3</v>
+      </c>
+      <c r="M6" s="8">
+        <f t="shared" si="1"/>
+        <v>0.36065493677846072</v>
+      </c>
+      <c r="N6" s="8">
+        <f t="shared" si="2"/>
+        <v>0.36253710775353737</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="8">
+        <v>0.16283259999999999</v>
+      </c>
+      <c r="E7" s="9">
+        <v>1.5103210000000001E-2</v>
+      </c>
+      <c r="F7" s="2">
+        <f t="shared" si="0"/>
+        <v>0.16529189495264598</v>
+      </c>
+      <c r="G7" s="8">
+        <f>F7/$F$8</f>
+        <v>0.16315218910370274</v>
+      </c>
+      <c r="I7" t="s">
+        <v>20</v>
+      </c>
+      <c r="J7" s="12">
+        <f>G6</f>
+        <v>0.12308832049207313</v>
+      </c>
+      <c r="K7" s="8">
+        <f>J7/SUM($J$5:$J$8)</f>
+        <v>0.27351747548102029</v>
+      </c>
+      <c r="L7" s="9">
+        <v>-9.2126670000000008E-3</v>
+      </c>
+      <c r="M7" s="8">
+        <f t="shared" si="1"/>
+        <v>0.27099765006073301</v>
+      </c>
+      <c r="N7" s="8">
+        <f t="shared" si="2"/>
+        <v>0.27241192131905662</v>
+      </c>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="F8" s="7">
+        <f>SUM(F4:F7)</f>
+        <v>1.0131147847950921</v>
+      </c>
+      <c r="I8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="12">
+        <f>G7</f>
+        <v>0.16315218910370274</v>
+      </c>
+      <c r="K8" s="8">
+        <f>J8/SUM($J$5:$J$8)</f>
+        <v>0.36254434786703127</v>
+      </c>
+      <c r="L8" s="9">
+        <v>1.686417E-3</v>
+      </c>
+      <c r="M8" s="8">
+        <f t="shared" si="1"/>
+        <v>0.36315574881852813</v>
+      </c>
+      <c r="N8" s="8">
+        <f t="shared" si="2"/>
+        <v>0.3650509709274059</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J9" s="6"/>
+      <c r="K9" s="6"/>
+      <c r="L9" s="6"/>
+      <c r="M9" s="9">
+        <f>SUM(M4:M8)</f>
+        <v>0.99480833565772198</v>
+      </c>
+      <c r="N9" s="6"/>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="19">
+        <f>SUMPRODUCT(L5:L8,K5:K8)</f>
+        <v>-5.1916643422782035E-3</v>
+      </c>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+    </row>
+    <row r="1048576" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G1048576" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
adjusted transaction cost calculation - bug corrected adjusted ausence of min_assets fallback bug
</commit_message>
<xml_diff>
--- a/tests/testthat/testdata/transaction_cost_calc.xlsx
+++ b/tests/testthat/testdata/transaction_cost_calc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paulo.fonteles\OneDrive - Sicoob\Renda Variável\Multifatorial 3.0\factoRverse\tests\testthat\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADCF3DFA-C9C7-4B81-B0A3-84EDA074AB1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9DA091A-94A1-420F-A28A-29DA00BFA837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20610" yWindow="-1065" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{0D95CC1D-80FD-4D8F-96FF-C13E93866E2C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{0D95CC1D-80FD-4D8F-96FF-C13E93866E2C}"/>
   </bookViews>
   <sheets>
     <sheet name="transaction_cost" sheetId="1" r:id="rId1"/>
@@ -142,12 +142,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.000000000000000%"/>
-    <numFmt numFmtId="169" formatCode="0.0000%"/>
+    <numFmt numFmtId="166" formatCode="0.000000000000000%"/>
+    <numFmt numFmtId="167" formatCode="0.0000%"/>
+    <numFmt numFmtId="169" formatCode="_-* #,##0.0000_-;\-* #,##0.0000_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="171" formatCode="0.0000"/>
   </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
@@ -640,7 +642,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1"/>
@@ -657,7 +659,7 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -676,7 +678,11 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1146,7 +1152,7 @@
         <f>E2-J2</f>
         <v>0.34800595112359295</v>
       </c>
-      <c r="L2">
+      <c r="L2" s="5">
         <f>K2*$L$8</f>
         <v>0.34800595112359295</v>
       </c>
@@ -1157,13 +1163,13 @@
       <c r="N2">
         <v>0.5</v>
       </c>
-      <c r="O2">
-        <f>ABS(L2*0.07)</f>
+      <c r="O2" s="21">
+        <f>ABS(L2)/$L$8*0.07</f>
         <v>2.4360416578651508E-2</v>
       </c>
       <c r="P2">
-        <f>ABS(M2)^N2*I2/2</f>
-        <v>0.25572780547838786</v>
+        <f>ABS(M2)^N2*I2/2*(ABS(L2)/$L$8)</f>
+        <v>8.8994798174255527E-2</v>
       </c>
       <c r="R2">
         <f>M2^N2*I2/2</f>
@@ -1205,7 +1211,7 @@
         <f>E3-J3</f>
         <v>-3.7167441940798018E-2</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="5">
         <f>K3*$L$8</f>
         <v>-3.7167441940798018E-2</v>
       </c>
@@ -1216,13 +1222,13 @@
       <c r="N3">
         <v>0.5</v>
       </c>
-      <c r="O3">
-        <f>ABS(L3*0.07)</f>
+      <c r="O3" s="21">
+        <f>ABS(L3)/$L$8*0.07</f>
         <v>2.6017209358558616E-3</v>
       </c>
       <c r="P3">
-        <f>ABS(M3)^N3*I3/2</f>
-        <v>6.1884465764165883E-3</v>
+        <f t="shared" ref="P3:P6" si="1">ABS(M3)^N3*I3/2*(ABS(L3)/$L$8)</f>
+        <v>2.3000872883269382E-4</v>
       </c>
       <c r="R3" t="e">
         <f>M3^N3*I3/2</f>
@@ -1264,7 +1270,7 @@
         <f>E4-J4</f>
         <v>-7.3671067241997013E-2</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="5">
         <f>K4*$L$8</f>
         <v>-7.3671067241997013E-2</v>
       </c>
@@ -1275,13 +1281,13 @@
       <c r="N4">
         <v>0.5</v>
       </c>
-      <c r="O4">
-        <f>ABS(L4*0.07)</f>
+      <c r="O4" s="21">
+        <f>ABS(L4)/$L$8*0.07</f>
         <v>5.1569747069397914E-3</v>
       </c>
       <c r="P4">
-        <f>ABS(M4)^N4*I4/2</f>
-        <v>0.15441254203649388</v>
+        <f t="shared" si="1"/>
+        <v>1.1375736767378231E-2</v>
       </c>
       <c r="R4" t="e">
         <f>M4^N4*I4/2</f>
@@ -1323,8 +1329,8 @@
         <f>E5-J5</f>
         <v>-3.7167441940798018E-2</v>
       </c>
-      <c r="L5">
-        <f t="shared" ref="L5:L6" si="1">K5*$L$8</f>
+      <c r="L5" s="5">
+        <f t="shared" ref="L5:L6" si="2">K5*$L$8</f>
         <v>-3.7167441940798018E-2</v>
       </c>
       <c r="M5" s="4">
@@ -1334,13 +1340,13 @@
       <c r="N5">
         <v>0.5</v>
       </c>
-      <c r="O5">
-        <f>ABS(L5*0.07)</f>
+      <c r="O5" s="21">
+        <f>ABS(L5)/$L$8*0.07</f>
         <v>2.6017209358558616E-3</v>
       </c>
       <c r="P5">
-        <f>ABS(M5)^N5*I5/2</f>
-        <v>3.0482090168348262E-2</v>
+        <f t="shared" si="1"/>
+        <v>1.1329413165662541E-3</v>
       </c>
       <c r="R5" t="e">
         <f>M5^N5*I5/2</f>
@@ -1382,8 +1388,8 @@
         <f>E6-J6</f>
         <v>-0.2</v>
       </c>
-      <c r="L6">
-        <f t="shared" si="1"/>
+      <c r="L6" s="5">
+        <f t="shared" si="2"/>
         <v>-0.2</v>
       </c>
       <c r="M6" s="5">
@@ -1393,13 +1399,13 @@
       <c r="N6">
         <v>0.5</v>
       </c>
-      <c r="O6">
-        <f>ABS(L6*0.07)</f>
+      <c r="O6" s="21">
+        <f>ABS(L6)/$L$8*0.07</f>
         <v>1.4000000000000002E-2</v>
       </c>
       <c r="P6">
-        <f>ABS(M6)^N6*I6/2</f>
-        <v>0.17266450280771806</v>
+        <f t="shared" si="1"/>
+        <v>3.4532900561543615E-2</v>
       </c>
       <c r="R6" t="e">
         <f>M6^N6*I6/2</f>
@@ -1407,11 +1413,21 @@
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K8">
+        <f t="array" ref="K8">SUM(ABS(K2:K6))/2</f>
+        <v>0.348005951123593</v>
+      </c>
       <c r="L8">
         <v>1</v>
       </c>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
+      <c r="O8" s="20">
+        <f>SUM(O2:O6)</f>
+        <v>4.8720833157303023E-2</v>
+      </c>
+      <c r="P8" s="20">
+        <f>SUM(P2:P6)</f>
+        <v>0.13626638554857631</v>
+      </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="O9" s="3"/>
@@ -1541,7 +1557,7 @@
         <v>1.9005850000000001E-2</v>
       </c>
       <c r="F5" s="2">
-        <f t="shared" ref="F5:G7" si="0">D5*(1+E5)</f>
+        <f t="shared" ref="F5:F7" si="0">D5*(1+E5)</f>
         <v>0.16592737197071</v>
       </c>
       <c r="G5" s="8">

</xml_diff>